<commit_message>
feat: add Vellore Winter 2026-27 course offerings
</commit_message>
<xml_diff>
--- a/util/report_vellore.xlsx
+++ b/util/report_vellore.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FFCS Data" sheetId="1" r:id="R9fc35fca98534dbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FFCS Data" sheetId="1" r:id="Re4b7e09a8c044a80"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,7 +485,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FFCSDataTable" displayName="FFCSDataTable" ref="A1:G146" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FFCSDataTable" displayName="FFCSDataTable" ref="A1:G179" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="CODE"/>
     <x:tableColumn id="2" name="TITLE"/>
@@ -4015,10 +4015,769 @@
         <x:v>SHILPI GUPTA</x:v>
       </x:c>
     </x:row>
+    <x:row r="147" ht="15" hidden="0" customHeight="1">
+      <x:c r="A147" s="61" t="str">
+        <x:v>BITE404E</x:v>
+      </x:c>
+      <x:c r="B147" s="62" t="str">
+        <x:v>Object Oriented Analysis and Design</x:v>
+      </x:c>
+      <x:c r="C147" s="62" t="str">
+        <x:v>ETH</x:v>
+      </x:c>
+      <x:c r="D147" s="107" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E147" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F147" s="62" t="str">
+        <x:v>G1</x:v>
+      </x:c>
+      <x:c r="G147" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" ht="15" hidden="0" customHeight="1">
+      <x:c r="A148" s="61" t="str">
+        <x:v>BITE404E</x:v>
+      </x:c>
+      <x:c r="B148" s="62" t="str">
+        <x:v>Object Oriented Analysis and Design</x:v>
+      </x:c>
+      <x:c r="C148" s="62" t="str">
+        <x:v>ELA</x:v>
+      </x:c>
+      <x:c r="D148" s="107" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E148" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F148" s="62" t="str">
+        <x:v>L55+L56</x:v>
+      </x:c>
+      <x:c r="G148" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="15" hidden="0" customHeight="1">
+      <x:c r="A149" s="61" t="str">
+        <x:v>BITE404E</x:v>
+      </x:c>
+      <x:c r="B149" s="62" t="str">
+        <x:v>Object Oriented Analysis and Design</x:v>
+      </x:c>
+      <x:c r="C149" s="62" t="str">
+        <x:v>ETH</x:v>
+      </x:c>
+      <x:c r="D149" s="107" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E149" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F149" s="62" t="str">
+        <x:v>G2</x:v>
+      </x:c>
+      <x:c r="G149" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="15" hidden="0" customHeight="1">
+      <x:c r="A150" s="61" t="str">
+        <x:v>BITE404E</x:v>
+      </x:c>
+      <x:c r="B150" s="62" t="str">
+        <x:v>Object Oriented Analysis and Design</x:v>
+      </x:c>
+      <x:c r="C150" s="62" t="str">
+        <x:v>ELA</x:v>
+      </x:c>
+      <x:c r="D150" s="107" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E150" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F150" s="62" t="str">
+        <x:v>L3+L4</x:v>
+      </x:c>
+      <x:c r="G150" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="15" hidden="0" customHeight="1">
+      <x:c r="A151" s="61" t="str">
+        <x:v>BITE404E</x:v>
+      </x:c>
+      <x:c r="B151" s="62" t="str">
+        <x:v>Object Oriented Analysis and Design</x:v>
+      </x:c>
+      <x:c r="C151" s="62" t="str">
+        <x:v>ELA</x:v>
+      </x:c>
+      <x:c r="D151" s="107" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E151" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F151" s="62" t="str">
+        <x:v>L45+L46</x:v>
+      </x:c>
+      <x:c r="G151" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="15" hidden="0" customHeight="1">
+      <x:c r="A152" s="61" t="str">
+        <x:v>BITE404E</x:v>
+      </x:c>
+      <x:c r="B152" s="62" t="str">
+        <x:v>Object Oriented Analysis and Design</x:v>
+      </x:c>
+      <x:c r="C152" s="62" t="str">
+        <x:v>ELA</x:v>
+      </x:c>
+      <x:c r="D152" s="107" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E152" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F152" s="62" t="str">
+        <x:v>L25+L26</x:v>
+      </x:c>
+      <x:c r="G152" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="15" hidden="0" customHeight="1">
+      <x:c r="A153" s="61" t="str">
+        <x:v>BITE311L</x:v>
+      </x:c>
+      <x:c r="B153" s="62" t="str">
+        <x:v>Human Computer Interaction</x:v>
+      </x:c>
+      <x:c r="C153" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D153" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E153" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F153" s="62" t="str">
+        <x:v>E1+TE1</x:v>
+      </x:c>
+      <x:c r="G153" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154" ht="15" hidden="0" customHeight="1">
+      <x:c r="A154" s="61" t="str">
+        <x:v>BITE311L</x:v>
+      </x:c>
+      <x:c r="B154" s="62" t="str">
+        <x:v>Human Computer Interaction</x:v>
+      </x:c>
+      <x:c r="C154" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D154" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E154" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F154" s="62" t="str">
+        <x:v>E2+TE2</x:v>
+      </x:c>
+      <x:c r="G154" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" ht="15" hidden="0" customHeight="1">
+      <x:c r="A155" s="61" t="str">
+        <x:v>BITE312E</x:v>
+      </x:c>
+      <x:c r="B155" s="62" t="str">
+        <x:v>Data Mining</x:v>
+      </x:c>
+      <x:c r="C155" s="62" t="str">
+        <x:v>ETH</x:v>
+      </x:c>
+      <x:c r="D155" s="107" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E155" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F155" s="62" t="str">
+        <x:v>G1</x:v>
+      </x:c>
+      <x:c r="G155" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156" ht="15" hidden="0" customHeight="1">
+      <x:c r="A156" s="61" t="str">
+        <x:v>BITE312E</x:v>
+      </x:c>
+      <x:c r="B156" s="62" t="str">
+        <x:v>Data Mining</x:v>
+      </x:c>
+      <x:c r="C156" s="62" t="str">
+        <x:v>ELA</x:v>
+      </x:c>
+      <x:c r="D156" s="107" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E156" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F156" s="62" t="str">
+        <x:v>L49+L50</x:v>
+      </x:c>
+      <x:c r="G156" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157" ht="15" hidden="0" customHeight="1">
+      <x:c r="A157" s="61" t="str">
+        <x:v>BITE312E</x:v>
+      </x:c>
+      <x:c r="B157" s="62" t="str">
+        <x:v>Data Mining</x:v>
+      </x:c>
+      <x:c r="C157" s="62" t="str">
+        <x:v>ETH</x:v>
+      </x:c>
+      <x:c r="D157" s="107" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E157" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F157" s="62" t="str">
+        <x:v>G2</x:v>
+      </x:c>
+      <x:c r="G157" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" ht="15" hidden="0" customHeight="1">
+      <x:c r="A158" s="61" t="str">
+        <x:v>BITE312E</x:v>
+      </x:c>
+      <x:c r="B158" s="62" t="str">
+        <x:v>Data Mining</x:v>
+      </x:c>
+      <x:c r="C158" s="62" t="str">
+        <x:v>ELA</x:v>
+      </x:c>
+      <x:c r="D158" s="107" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E158" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F158" s="62" t="str">
+        <x:v>L11+L12</x:v>
+      </x:c>
+      <x:c r="G158" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159" ht="15" hidden="0" customHeight="1">
+      <x:c r="A159" s="61" t="str">
+        <x:v>BITE312E</x:v>
+      </x:c>
+      <x:c r="B159" s="62" t="str">
+        <x:v>Data Mining</x:v>
+      </x:c>
+      <x:c r="C159" s="62" t="str">
+        <x:v>ELA</x:v>
+      </x:c>
+      <x:c r="D159" s="107" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E159" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F159" s="62" t="str">
+        <x:v>L51+L52</x:v>
+      </x:c>
+      <x:c r="G159" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="15" hidden="0" customHeight="1">
+      <x:c r="A160" s="61" t="str">
+        <x:v>BITE312E</x:v>
+      </x:c>
+      <x:c r="B160" s="62" t="str">
+        <x:v>Data Mining</x:v>
+      </x:c>
+      <x:c r="C160" s="62" t="str">
+        <x:v>ELA</x:v>
+      </x:c>
+      <x:c r="D160" s="107" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E160" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F160" s="62" t="str">
+        <x:v>L1+L2</x:v>
+      </x:c>
+      <x:c r="G160" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161" ht="15" hidden="0" customHeight="1">
+      <x:c r="A161" s="61" t="str">
+        <x:v>BITE401L</x:v>
+      </x:c>
+      <x:c r="B161" s="62" t="str">
+        <x:v>Network and Information Security</x:v>
+      </x:c>
+      <x:c r="C161" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D161" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E161" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F161" s="62" t="str">
+        <x:v>A1+TA1</x:v>
+      </x:c>
+      <x:c r="G161" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="15" hidden="0" customHeight="1">
+      <x:c r="A162" s="61" t="str">
+        <x:v>BITE401L</x:v>
+      </x:c>
+      <x:c r="B162" s="62" t="str">
+        <x:v>Network and Information Security</x:v>
+      </x:c>
+      <x:c r="C162" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D162" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E162" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F162" s="62" t="str">
+        <x:v>A2+TA2</x:v>
+      </x:c>
+      <x:c r="G162" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" ht="15" hidden="0" customHeight="1">
+      <x:c r="A163" s="61" t="str">
+        <x:v>BITE402L</x:v>
+      </x:c>
+      <x:c r="B163" s="62" t="str">
+        <x:v>Distributed Computing</x:v>
+      </x:c>
+      <x:c r="C163" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D163" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E163" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F163" s="62" t="str">
+        <x:v>B1+TB1</x:v>
+      </x:c>
+      <x:c r="G163" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="15" hidden="0" customHeight="1">
+      <x:c r="A164" s="61" t="str">
+        <x:v>BITE402L</x:v>
+      </x:c>
+      <x:c r="B164" s="62" t="str">
+        <x:v>Distributed Computing</x:v>
+      </x:c>
+      <x:c r="C164" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D164" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E164" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F164" s="62" t="str">
+        <x:v>B2+TB2</x:v>
+      </x:c>
+      <x:c r="G164" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="15" hidden="0" customHeight="1">
+      <x:c r="A165" s="61" t="str">
+        <x:v>BITE405L</x:v>
+      </x:c>
+      <x:c r="B165" s="62" t="str">
+        <x:v>Soft Computing</x:v>
+      </x:c>
+      <x:c r="C165" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D165" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E165" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F165" s="62" t="str">
+        <x:v>C1+TC1</x:v>
+      </x:c>
+      <x:c r="G165" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="15" hidden="0" customHeight="1">
+      <x:c r="A166" s="61" t="str">
+        <x:v>BITE405L</x:v>
+      </x:c>
+      <x:c r="B166" s="62" t="str">
+        <x:v>Soft Computing</x:v>
+      </x:c>
+      <x:c r="C166" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D166" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E166" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F166" s="62" t="str">
+        <x:v>C2+TC2</x:v>
+      </x:c>
+      <x:c r="G166" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="15" hidden="0" customHeight="1">
+      <x:c r="A167" s="61" t="str">
+        <x:v>BITE409L</x:v>
+      </x:c>
+      <x:c r="B167" s="62" t="str">
+        <x:v>Mobile Application Development</x:v>
+      </x:c>
+      <x:c r="C167" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D167" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E167" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F167" s="62" t="str">
+        <x:v>C1+TC1</x:v>
+      </x:c>
+      <x:c r="G167" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="15" hidden="0" customHeight="1">
+      <x:c r="A168" s="61" t="str">
+        <x:v>BITE409L</x:v>
+      </x:c>
+      <x:c r="B168" s="62" t="str">
+        <x:v>Mobile Application Development</x:v>
+      </x:c>
+      <x:c r="C168" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D168" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E168" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F168" s="62" t="str">
+        <x:v>C2+TC2</x:v>
+      </x:c>
+      <x:c r="G168" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="15" hidden="0" customHeight="1">
+      <x:c r="A169" s="61" t="str">
+        <x:v>BITE410L</x:v>
+      </x:c>
+      <x:c r="B169" s="62" t="str">
+        <x:v>Machine Learning</x:v>
+      </x:c>
+      <x:c r="C169" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D169" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E169" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F169" s="62" t="str">
+        <x:v>E1+TE1</x:v>
+      </x:c>
+      <x:c r="G169" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="15" hidden="0" customHeight="1">
+      <x:c r="A170" s="61" t="str">
+        <x:v>BITE410L</x:v>
+      </x:c>
+      <x:c r="B170" s="62" t="str">
+        <x:v>Machine Learning</x:v>
+      </x:c>
+      <x:c r="C170" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D170" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E170" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F170" s="62" t="str">
+        <x:v>E2+TE2</x:v>
+      </x:c>
+      <x:c r="G170" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" ht="15" hidden="0" customHeight="1">
+      <x:c r="A171" s="61" t="str">
+        <x:v>BITE411L</x:v>
+      </x:c>
+      <x:c r="B171" s="62" t="str">
+        <x:v>Big Data Analytics</x:v>
+      </x:c>
+      <x:c r="C171" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D171" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E171" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F171" s="62" t="str">
+        <x:v>D1+TD1</x:v>
+      </x:c>
+      <x:c r="G171" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172" ht="15" hidden="0" customHeight="1">
+      <x:c r="A172" s="61" t="str">
+        <x:v>BITE411L</x:v>
+      </x:c>
+      <x:c r="B172" s="62" t="str">
+        <x:v>Big Data Analytics</x:v>
+      </x:c>
+      <x:c r="C172" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D172" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E172" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F172" s="62" t="str">
+        <x:v>D2+TD2</x:v>
+      </x:c>
+      <x:c r="G172" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" ht="15" hidden="0" customHeight="1">
+      <x:c r="A173" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B173" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C173" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D173" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E173" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F173" s="62" t="str">
+        <x:v>F1</x:v>
+      </x:c>
+      <x:c r="G173" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="15" hidden="0" customHeight="1">
+      <x:c r="A174" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B174" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C174" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D174" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E174" s="62" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+      <x:c r="F174" s="62" t="str">
+        <x:v>F2</x:v>
+      </x:c>
+      <x:c r="G174" s="63" t="str">
+        <x:v>Not announced</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" ht="15" hidden="0" customHeight="1">
+      <x:c r="A175" s="61" t="str">
+        <x:v>BITE301L</x:v>
+      </x:c>
+      <x:c r="B175" s="62" t="str">
+        <x:v>Computer Architecture and Organization</x:v>
+      </x:c>
+      <x:c r="C175" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D175" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E175" s="62" t="str">
+        <x:v>PRP426</x:v>
+      </x:c>
+      <x:c r="F175" s="62" t="str">
+        <x:v>A1+TA1</x:v>
+      </x:c>
+      <x:c r="G175" s="63" t="str">
+        <x:v>KARPAGAM S</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176" ht="15" hidden="0" customHeight="1">
+      <x:c r="A176" s="61" t="str">
+        <x:v>BCSE102L</x:v>
+      </x:c>
+      <x:c r="B176" s="62" t="str">
+        <x:v>Structured and Object-Oriented Programming</x:v>
+      </x:c>
+      <x:c r="C176" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D176" s="107" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E176" s="62" t="str">
+        <x:v>PRP330</x:v>
+      </x:c>
+      <x:c r="F176" s="62" t="str">
+        <x:v>D1</x:v>
+      </x:c>
+      <x:c r="G176" s="63" t="str">
+        <x:v>SUKANTA GHOSH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="15" hidden="0" customHeight="1">
+      <x:c r="A177" s="61" t="str">
+        <x:v>BCSE102L</x:v>
+      </x:c>
+      <x:c r="B177" s="62" t="str">
+        <x:v>Structured and Object-Oriented Programming</x:v>
+      </x:c>
+      <x:c r="C177" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D177" s="107" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E177" s="62" t="str">
+        <x:v>PRP330</x:v>
+      </x:c>
+      <x:c r="F177" s="62" t="str">
+        <x:v>D2</x:v>
+      </x:c>
+      <x:c r="G177" s="63" t="str">
+        <x:v>SUKANTA GHOSH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="15" hidden="0" customHeight="1">
+      <x:c r="A178" s="61" t="str">
+        <x:v>BCSE102P</x:v>
+      </x:c>
+      <x:c r="B178" s="62" t="str">
+        <x:v>Structured and Object-Oriented Programming Lab</x:v>
+      </x:c>
+      <x:c r="C178" s="62" t="str">
+        <x:v>LO</x:v>
+      </x:c>
+      <x:c r="D178" s="107" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E178" s="62" t="str">
+        <x:v>PRP347</x:v>
+      </x:c>
+      <x:c r="F178" s="62" t="str">
+        <x:v>L39+L40+L55+L56</x:v>
+      </x:c>
+      <x:c r="G178" s="63" t="str">
+        <x:v>SUKANTA GHOSH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="15" hidden="0" customHeight="1">
+      <x:c r="A179" s="61" t="str">
+        <x:v>BCSE102P</x:v>
+      </x:c>
+      <x:c r="B179" s="62" t="str">
+        <x:v>Structured and Object-Oriented Programming Lab</x:v>
+      </x:c>
+      <x:c r="C179" s="62" t="str">
+        <x:v>LO</x:v>
+      </x:c>
+      <x:c r="D179" s="107" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E179" s="62" t="str">
+        <x:v>PRP138</x:v>
+      </x:c>
+      <x:c r="F179" s="62" t="str">
+        <x:v>L13+L14+L27+L28</x:v>
+      </x:c>
+      <x:c r="G179" s="63" t="str">
+        <x:v>SUKANTA GHOSH</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14bb34c55d274206"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9479282cab684baf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: complete Vellore allocations with verified VTOP data
</commit_message>
<xml_diff>
--- a/util/report_vellore.xlsx
+++ b/util/report_vellore.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FFCS Data" sheetId="1" r:id="Re4b7e09a8c044a80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FFCS Data" sheetId="1" r:id="R12e28a09f306488b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,7 +485,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FFCSDataTable" displayName="FFCSDataTable" ref="A1:G179" headerRowCount="1" totalsRowCount="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FFCSDataTable" displayName="FFCSDataTable" ref="A1:G259" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="CODE"/>
     <x:tableColumn id="2" name="TITLE"/>
@@ -4017,140 +4017,140 @@
     </x:row>
     <x:row r="147" ht="15" hidden="0" customHeight="1">
       <x:c r="A147" s="61" t="str">
-        <x:v>BITE404E</x:v>
+        <x:v>BITE301L</x:v>
       </x:c>
       <x:c r="B147" s="62" t="str">
-        <x:v>Object Oriented Analysis and Design</x:v>
+        <x:v>Computer Architecture and Organization</x:v>
       </x:c>
       <x:c r="C147" s="62" t="str">
-        <x:v>ETH</x:v>
+        <x:v>TH</x:v>
       </x:c>
       <x:c r="D147" s="107" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E147" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>PRP426</x:v>
       </x:c>
       <x:c r="F147" s="62" t="str">
-        <x:v>G1</x:v>
+        <x:v>A1+TA1</x:v>
       </x:c>
       <x:c r="G147" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>KARPAGAM S</x:v>
       </x:c>
     </x:row>
     <x:row r="148" ht="15" hidden="0" customHeight="1">
       <x:c r="A148" s="61" t="str">
-        <x:v>BITE404E</x:v>
+        <x:v>BCSE102L</x:v>
       </x:c>
       <x:c r="B148" s="62" t="str">
-        <x:v>Object Oriented Analysis and Design</x:v>
+        <x:v>Structured and Object-Oriented Programming</x:v>
       </x:c>
       <x:c r="C148" s="62" t="str">
-        <x:v>ELA</x:v>
+        <x:v>TH</x:v>
       </x:c>
       <x:c r="D148" s="107" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E148" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>PRP330</x:v>
       </x:c>
       <x:c r="F148" s="62" t="str">
-        <x:v>L55+L56</x:v>
+        <x:v>D1</x:v>
       </x:c>
       <x:c r="G148" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SUKANTA GHOSH</x:v>
       </x:c>
     </x:row>
     <x:row r="149" ht="15" hidden="0" customHeight="1">
       <x:c r="A149" s="61" t="str">
-        <x:v>BITE404E</x:v>
+        <x:v>BCSE102L</x:v>
       </x:c>
       <x:c r="B149" s="62" t="str">
-        <x:v>Object Oriented Analysis and Design</x:v>
+        <x:v>Structured and Object-Oriented Programming</x:v>
       </x:c>
       <x:c r="C149" s="62" t="str">
-        <x:v>ETH</x:v>
+        <x:v>TH</x:v>
       </x:c>
       <x:c r="D149" s="107" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E149" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>PRP330</x:v>
       </x:c>
       <x:c r="F149" s="62" t="str">
-        <x:v>G2</x:v>
+        <x:v>D2</x:v>
       </x:c>
       <x:c r="G149" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SUKANTA GHOSH</x:v>
       </x:c>
     </x:row>
     <x:row r="150" ht="15" hidden="0" customHeight="1">
       <x:c r="A150" s="61" t="str">
-        <x:v>BITE404E</x:v>
+        <x:v>BCSE102P</x:v>
       </x:c>
       <x:c r="B150" s="62" t="str">
-        <x:v>Object Oriented Analysis and Design</x:v>
+        <x:v>Structured and Object-Oriented Programming Lab</x:v>
       </x:c>
       <x:c r="C150" s="62" t="str">
-        <x:v>ELA</x:v>
+        <x:v>LO</x:v>
       </x:c>
       <x:c r="D150" s="107" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E150" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>PRP347</x:v>
       </x:c>
       <x:c r="F150" s="62" t="str">
-        <x:v>L3+L4</x:v>
+        <x:v>L39+L40+L55+L56</x:v>
       </x:c>
       <x:c r="G150" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SUKANTA GHOSH</x:v>
       </x:c>
     </x:row>
     <x:row r="151" ht="15" hidden="0" customHeight="1">
       <x:c r="A151" s="61" t="str">
-        <x:v>BITE404E</x:v>
+        <x:v>BCSE102P</x:v>
       </x:c>
       <x:c r="B151" s="62" t="str">
-        <x:v>Object Oriented Analysis and Design</x:v>
+        <x:v>Structured and Object-Oriented Programming Lab</x:v>
       </x:c>
       <x:c r="C151" s="62" t="str">
-        <x:v>ELA</x:v>
+        <x:v>LO</x:v>
       </x:c>
       <x:c r="D151" s="107" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E151" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>PRP138</x:v>
       </x:c>
       <x:c r="F151" s="62" t="str">
-        <x:v>L45+L46</x:v>
+        <x:v>L13+L14+L27+L28</x:v>
       </x:c>
       <x:c r="G151" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SUKANTA GHOSH</x:v>
       </x:c>
     </x:row>
     <x:row r="152" ht="15" hidden="0" customHeight="1">
       <x:c r="A152" s="61" t="str">
-        <x:v>BITE404E</x:v>
+        <x:v>BITE311L</x:v>
       </x:c>
       <x:c r="B152" s="62" t="str">
-        <x:v>Object Oriented Analysis and Design</x:v>
+        <x:v>Human Computer Interaction</x:v>
       </x:c>
       <x:c r="C152" s="62" t="str">
-        <x:v>ELA</x:v>
+        <x:v>TH</x:v>
       </x:c>
       <x:c r="D152" s="107" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E152" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT823</x:v>
       </x:c>
       <x:c r="F152" s="62" t="str">
-        <x:v>L25+L26</x:v>
+        <x:v>E2+TE2</x:v>
       </x:c>
       <x:c r="G152" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>AASEEGHA M D</x:v>
       </x:c>
     </x:row>
     <x:row r="153" ht="15" hidden="0" customHeight="1">
@@ -4167,13 +4167,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E153" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT803</x:v>
       </x:c>
       <x:c r="F153" s="62" t="str">
-        <x:v>E1+TE1</x:v>
+        <x:v>E2+TE2</x:v>
       </x:c>
       <x:c r="G153" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>BHUVANESWARI M S</x:v>
       </x:c>
     </x:row>
     <x:row r="154" ht="15" hidden="0" customHeight="1">
@@ -4190,36 +4190,36 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E154" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJTG24</x:v>
       </x:c>
       <x:c r="F154" s="62" t="str">
-        <x:v>E2+TE2</x:v>
+        <x:v>E1+TE1</x:v>
       </x:c>
       <x:c r="G154" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>JENILA VINCENT M</x:v>
       </x:c>
     </x:row>
     <x:row r="155" ht="15" hidden="0" customHeight="1">
       <x:c r="A155" s="61" t="str">
-        <x:v>BITE312E</x:v>
+        <x:v>BITE311L</x:v>
       </x:c>
       <x:c r="B155" s="62" t="str">
-        <x:v>Data Mining</x:v>
+        <x:v>Human Computer Interaction</x:v>
       </x:c>
       <x:c r="C155" s="62" t="str">
-        <x:v>ETH</x:v>
+        <x:v>TH</x:v>
       </x:c>
       <x:c r="D155" s="107" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E155" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT824</x:v>
       </x:c>
       <x:c r="F155" s="62" t="str">
-        <x:v>G1</x:v>
+        <x:v>E1+TE1</x:v>
       </x:c>
       <x:c r="G155" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>DEEPA P</x:v>
       </x:c>
     </x:row>
     <x:row r="156" ht="15" hidden="0" customHeight="1">
@@ -4230,19 +4230,19 @@
         <x:v>Data Mining</x:v>
       </x:c>
       <x:c r="C156" s="62" t="str">
-        <x:v>ELA</x:v>
+        <x:v>ETH</x:v>
       </x:c>
       <x:c r="D156" s="107" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E156" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT824</x:v>
       </x:c>
       <x:c r="F156" s="62" t="str">
-        <x:v>L49+L50</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="G156" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SENTHILKUMAR N C</x:v>
       </x:c>
     </x:row>
     <x:row r="157" ht="15" hidden="0" customHeight="1">
@@ -4253,19 +4253,19 @@
         <x:v>Data Mining</x:v>
       </x:c>
       <x:c r="C157" s="62" t="str">
-        <x:v>ETH</x:v>
+        <x:v>ELA</x:v>
       </x:c>
       <x:c r="D157" s="107" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E157" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJTG20</x:v>
       </x:c>
       <x:c r="F157" s="62" t="str">
-        <x:v>G2</x:v>
+        <x:v>L49+L50</x:v>
       </x:c>
       <x:c r="G157" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>PRABHANANTHA KUMAR M</x:v>
       </x:c>
     </x:row>
     <x:row r="158" ht="15" hidden="0" customHeight="1">
@@ -4276,19 +4276,19 @@
         <x:v>Data Mining</x:v>
       </x:c>
       <x:c r="C158" s="62" t="str">
-        <x:v>ELA</x:v>
+        <x:v>ETH</x:v>
       </x:c>
       <x:c r="D158" s="107" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E158" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT105</x:v>
       </x:c>
       <x:c r="F158" s="62" t="str">
-        <x:v>L11+L12</x:v>
+        <x:v>G1</x:v>
       </x:c>
       <x:c r="G158" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>YOGA RAJA C A</x:v>
       </x:c>
     </x:row>
     <x:row r="159" ht="15" hidden="0" customHeight="1">
@@ -4305,13 +4305,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E159" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJTG20</x:v>
       </x:c>
       <x:c r="F159" s="62" t="str">
-        <x:v>L51+L52</x:v>
+        <x:v>L1+L2</x:v>
       </x:c>
       <x:c r="G159" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>JAI KUMARAN</x:v>
       </x:c>
     </x:row>
     <x:row r="160" ht="15" hidden="0" customHeight="1">
@@ -4322,280 +4322,280 @@
         <x:v>Data Mining</x:v>
       </x:c>
       <x:c r="C160" s="62" t="str">
-        <x:v>ELA</x:v>
+        <x:v>ETH</x:v>
       </x:c>
       <x:c r="D160" s="107" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E160" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>PRP230</x:v>
       </x:c>
       <x:c r="F160" s="62" t="str">
-        <x:v>L1+L2</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="G160" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>JAI KUMARAN</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="15" hidden="0" customHeight="1">
       <x:c r="A161" s="61" t="str">
-        <x:v>BITE401L</x:v>
+        <x:v>BITE312E</x:v>
       </x:c>
       <x:c r="B161" s="62" t="str">
-        <x:v>Network and Information Security</x:v>
+        <x:v>Data Mining</x:v>
       </x:c>
       <x:c r="C161" s="62" t="str">
-        <x:v>TH</x:v>
+        <x:v>ETH</x:v>
       </x:c>
       <x:c r="D161" s="107" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E161" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT712</x:v>
       </x:c>
       <x:c r="F161" s="62" t="str">
-        <x:v>A1+TA1</x:v>
+        <x:v>G1</x:v>
       </x:c>
       <x:c r="G161" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>PRABHANANTHA KUMAR M</x:v>
       </x:c>
     </x:row>
     <x:row r="162" ht="15" hidden="0" customHeight="1">
       <x:c r="A162" s="61" t="str">
-        <x:v>BITE401L</x:v>
+        <x:v>BITE312E</x:v>
       </x:c>
       <x:c r="B162" s="62" t="str">
-        <x:v>Network and Information Security</x:v>
+        <x:v>Data Mining</x:v>
       </x:c>
       <x:c r="C162" s="62" t="str">
-        <x:v>TH</x:v>
+        <x:v>ELA</x:v>
       </x:c>
       <x:c r="D162" s="107" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E162" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJTG20</x:v>
       </x:c>
       <x:c r="F162" s="62" t="str">
-        <x:v>A2+TA2</x:v>
+        <x:v>L51+L52</x:v>
       </x:c>
       <x:c r="G162" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>YOGA RAJA C A</x:v>
       </x:c>
     </x:row>
     <x:row r="163" ht="15" hidden="0" customHeight="1">
       <x:c r="A163" s="61" t="str">
-        <x:v>BITE402L</x:v>
+        <x:v>BITE312E</x:v>
       </x:c>
       <x:c r="B163" s="62" t="str">
-        <x:v>Distributed Computing</x:v>
+        <x:v>Data Mining</x:v>
       </x:c>
       <x:c r="C163" s="62" t="str">
-        <x:v>TH</x:v>
+        <x:v>ELA</x:v>
       </x:c>
       <x:c r="D163" s="107" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E163" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJTG20</x:v>
       </x:c>
       <x:c r="F163" s="62" t="str">
-        <x:v>B1+TB1</x:v>
+        <x:v>L11+L12</x:v>
       </x:c>
       <x:c r="G163" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SENTHILKUMAR N C</x:v>
       </x:c>
     </x:row>
     <x:row r="164" ht="15" hidden="0" customHeight="1">
       <x:c r="A164" s="61" t="str">
-        <x:v>BITE402L</x:v>
+        <x:v>BITE404E</x:v>
       </x:c>
       <x:c r="B164" s="62" t="str">
-        <x:v>Distributed Computing</x:v>
+        <x:v>Object Oriented Analysis and Design</x:v>
       </x:c>
       <x:c r="C164" s="62" t="str">
-        <x:v>TH</x:v>
+        <x:v>ELA</x:v>
       </x:c>
       <x:c r="D164" s="107" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E164" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT219</x:v>
       </x:c>
       <x:c r="F164" s="62" t="str">
-        <x:v>B2+TB2</x:v>
+        <x:v>L45+L46</x:v>
       </x:c>
       <x:c r="G164" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SRIVATHSAVA M</x:v>
       </x:c>
     </x:row>
     <x:row r="165" ht="15" hidden="0" customHeight="1">
       <x:c r="A165" s="61" t="str">
-        <x:v>BITE405L</x:v>
+        <x:v>BITE404E</x:v>
       </x:c>
       <x:c r="B165" s="62" t="str">
-        <x:v>Soft Computing</x:v>
+        <x:v>Object Oriented Analysis and Design</x:v>
       </x:c>
       <x:c r="C165" s="62" t="str">
-        <x:v>TH</x:v>
+        <x:v>ELA</x:v>
       </x:c>
       <x:c r="D165" s="107" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E165" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJTG20</x:v>
       </x:c>
       <x:c r="F165" s="62" t="str">
-        <x:v>C1+TC1</x:v>
+        <x:v>L3+L4</x:v>
       </x:c>
       <x:c r="G165" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SRIVATHSAVA M</x:v>
       </x:c>
     </x:row>
     <x:row r="166" ht="15" hidden="0" customHeight="1">
       <x:c r="A166" s="61" t="str">
-        <x:v>BITE405L</x:v>
+        <x:v>BITE404E</x:v>
       </x:c>
       <x:c r="B166" s="62" t="str">
-        <x:v>Soft Computing</x:v>
+        <x:v>Object Oriented Analysis and Design</x:v>
       </x:c>
       <x:c r="C166" s="62" t="str">
-        <x:v>TH</x:v>
+        <x:v>ELA</x:v>
       </x:c>
       <x:c r="D166" s="107" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E166" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT219</x:v>
       </x:c>
       <x:c r="F166" s="62" t="str">
-        <x:v>C2+TC2</x:v>
+        <x:v>L25+L26</x:v>
       </x:c>
       <x:c r="G166" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SUJANA M</x:v>
       </x:c>
     </x:row>
     <x:row r="167" ht="15" hidden="0" customHeight="1">
       <x:c r="A167" s="61" t="str">
-        <x:v>BITE409L</x:v>
+        <x:v>BITE404E</x:v>
       </x:c>
       <x:c r="B167" s="62" t="str">
-        <x:v>Mobile Application Development</x:v>
+        <x:v>Object Oriented Analysis and Design</x:v>
       </x:c>
       <x:c r="C167" s="62" t="str">
-        <x:v>TH</x:v>
+        <x:v>ETH</x:v>
       </x:c>
       <x:c r="D167" s="107" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E167" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT709</x:v>
       </x:c>
       <x:c r="F167" s="62" t="str">
-        <x:v>C1+TC1</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="G167" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SRIVATHSAVA M</x:v>
       </x:c>
     </x:row>
     <x:row r="168" ht="15" hidden="0" customHeight="1">
       <x:c r="A168" s="61" t="str">
-        <x:v>BITE409L</x:v>
+        <x:v>BITE404E</x:v>
       </x:c>
       <x:c r="B168" s="62" t="str">
-        <x:v>Mobile Application Development</x:v>
+        <x:v>Object Oriented Analysis and Design</x:v>
       </x:c>
       <x:c r="C168" s="62" t="str">
-        <x:v>TH</x:v>
+        <x:v>ETH</x:v>
       </x:c>
       <x:c r="D168" s="107" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E168" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT711</x:v>
       </x:c>
       <x:c r="F168" s="62" t="str">
-        <x:v>C2+TC2</x:v>
+        <x:v>G1</x:v>
       </x:c>
       <x:c r="G168" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SUGANYA A</x:v>
       </x:c>
     </x:row>
     <x:row r="169" ht="15" hidden="0" customHeight="1">
       <x:c r="A169" s="61" t="str">
-        <x:v>BITE410L</x:v>
+        <x:v>BITE404E</x:v>
       </x:c>
       <x:c r="B169" s="62" t="str">
-        <x:v>Machine Learning</x:v>
+        <x:v>Object Oriented Analysis and Design</x:v>
       </x:c>
       <x:c r="C169" s="62" t="str">
-        <x:v>TH</x:v>
+        <x:v>ETH</x:v>
       </x:c>
       <x:c r="D169" s="107" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E169" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>PRP426</x:v>
       </x:c>
       <x:c r="F169" s="62" t="str">
-        <x:v>E1+TE1</x:v>
+        <x:v>G1</x:v>
       </x:c>
       <x:c r="G169" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SRIVATHSAVA M</x:v>
       </x:c>
     </x:row>
     <x:row r="170" ht="15" hidden="0" customHeight="1">
       <x:c r="A170" s="61" t="str">
-        <x:v>BITE410L</x:v>
+        <x:v>BITE404E</x:v>
       </x:c>
       <x:c r="B170" s="62" t="str">
-        <x:v>Machine Learning</x:v>
+        <x:v>Object Oriented Analysis and Design</x:v>
       </x:c>
       <x:c r="C170" s="62" t="str">
-        <x:v>TH</x:v>
+        <x:v>ETH</x:v>
       </x:c>
       <x:c r="D170" s="107" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E170" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT711</x:v>
       </x:c>
       <x:c r="F170" s="62" t="str">
-        <x:v>E2+TE2</x:v>
+        <x:v>G2</x:v>
       </x:c>
       <x:c r="G170" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SUJANA M</x:v>
       </x:c>
     </x:row>
     <x:row r="171" ht="15" hidden="0" customHeight="1">
       <x:c r="A171" s="61" t="str">
-        <x:v>BITE411L</x:v>
+        <x:v>BITE404E</x:v>
       </x:c>
       <x:c r="B171" s="62" t="str">
-        <x:v>Big Data Analytics</x:v>
+        <x:v>Object Oriented Analysis and Design</x:v>
       </x:c>
       <x:c r="C171" s="62" t="str">
-        <x:v>TH</x:v>
+        <x:v>ELA</x:v>
       </x:c>
       <x:c r="D171" s="107" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E171" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT122</x:v>
       </x:c>
       <x:c r="F171" s="62" t="str">
-        <x:v>D1+TD1</x:v>
+        <x:v>L55+L56</x:v>
       </x:c>
       <x:c r="G171" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SUGANYA A</x:v>
       </x:c>
     </x:row>
     <x:row r="172" ht="15" hidden="0" customHeight="1">
       <x:c r="A172" s="61" t="str">
-        <x:v>BITE411L</x:v>
+        <x:v>BITE405L</x:v>
       </x:c>
       <x:c r="B172" s="62" t="str">
-        <x:v>Big Data Analytics</x:v>
+        <x:v>Soft Computing</x:v>
       </x:c>
       <x:c r="C172" s="62" t="str">
         <x:v>TH</x:v>
@@ -4604,21 +4604,21 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E172" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT211</x:v>
       </x:c>
       <x:c r="F172" s="62" t="str">
-        <x:v>D2+TD2</x:v>
+        <x:v>C2+TC2</x:v>
       </x:c>
       <x:c r="G172" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>BRIJENDRA SINGH</x:v>
       </x:c>
     </x:row>
     <x:row r="173" ht="15" hidden="0" customHeight="1">
       <x:c r="A173" s="61" t="str">
-        <x:v>BSTS302P</x:v>
+        <x:v>BITE405L</x:v>
       </x:c>
       <x:c r="B173" s="62" t="str">
-        <x:v>Advanced Competitive Coding - II</x:v>
+        <x:v>Soft Computing</x:v>
       </x:c>
       <x:c r="C173" s="62" t="str">
         <x:v>TH</x:v>
@@ -4627,21 +4627,21 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E173" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT825</x:v>
       </x:c>
       <x:c r="F173" s="62" t="str">
-        <x:v>F1</x:v>
+        <x:v>C2+TC2</x:v>
       </x:c>
       <x:c r="G173" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>NEELU KHARE</x:v>
       </x:c>
     </x:row>
     <x:row r="174" ht="15" hidden="0" customHeight="1">
       <x:c r="A174" s="61" t="str">
-        <x:v>BSTS302P</x:v>
+        <x:v>BITE405L</x:v>
       </x:c>
       <x:c r="B174" s="62" t="str">
-        <x:v>Advanced Competitive Coding - II</x:v>
+        <x:v>Soft Computing</x:v>
       </x:c>
       <x:c r="C174" s="62" t="str">
         <x:v>TH</x:v>
@@ -4650,21 +4650,21 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E174" s="62" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>SJT807</x:v>
       </x:c>
       <x:c r="F174" s="62" t="str">
-        <x:v>F2</x:v>
+        <x:v>C1+TC1</x:v>
       </x:c>
       <x:c r="G174" s="63" t="str">
-        <x:v>Not announced</x:v>
+        <x:v>CHIRANJI LAL CHOWDHARY</x:v>
       </x:c>
     </x:row>
     <x:row r="175" ht="15" hidden="0" customHeight="1">
       <x:c r="A175" s="61" t="str">
-        <x:v>BITE301L</x:v>
+        <x:v>BITE405L</x:v>
       </x:c>
       <x:c r="B175" s="62" t="str">
-        <x:v>Computer Architecture and Organization</x:v>
+        <x:v>Soft Computing</x:v>
       </x:c>
       <x:c r="C175" s="62" t="str">
         <x:v>TH</x:v>
@@ -4673,111 +4673,1951 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E175" s="62" t="str">
-        <x:v>PRP426</x:v>
+        <x:v>SJT825</x:v>
       </x:c>
       <x:c r="F175" s="62" t="str">
-        <x:v>A1+TA1</x:v>
+        <x:v>C1+TC1</x:v>
       </x:c>
       <x:c r="G175" s="63" t="str">
-        <x:v>KARPAGAM S</x:v>
+        <x:v>NEELU KHARE</x:v>
       </x:c>
     </x:row>
     <x:row r="176" ht="15" hidden="0" customHeight="1">
       <x:c r="A176" s="61" t="str">
-        <x:v>BCSE102L</x:v>
+        <x:v>BITE409L</x:v>
       </x:c>
       <x:c r="B176" s="62" t="str">
-        <x:v>Structured and Object-Oriented Programming</x:v>
+        <x:v>Mobile Application Development</x:v>
       </x:c>
       <x:c r="C176" s="62" t="str">
         <x:v>TH</x:v>
       </x:c>
       <x:c r="D176" s="107" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E176" s="62" t="str">
-        <x:v>PRP330</x:v>
+        <x:v>SJT823</x:v>
       </x:c>
       <x:c r="F176" s="62" t="str">
-        <x:v>D1</x:v>
+        <x:v>C1+TC1</x:v>
       </x:c>
       <x:c r="G176" s="63" t="str">
-        <x:v>SUKANTA GHOSH</x:v>
+        <x:v>SENTHIL KUMARAN U</x:v>
       </x:c>
     </x:row>
     <x:row r="177" ht="15" hidden="0" customHeight="1">
       <x:c r="A177" s="61" t="str">
-        <x:v>BCSE102L</x:v>
+        <x:v>BITE409L</x:v>
       </x:c>
       <x:c r="B177" s="62" t="str">
-        <x:v>Structured and Object-Oriented Programming</x:v>
+        <x:v>Mobile Application Development</x:v>
       </x:c>
       <x:c r="C177" s="62" t="str">
         <x:v>TH</x:v>
       </x:c>
       <x:c r="D177" s="107" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E177" s="62" t="str">
-        <x:v>PRP330</x:v>
+        <x:v>SJT824</x:v>
       </x:c>
       <x:c r="F177" s="62" t="str">
-        <x:v>D2</x:v>
+        <x:v>C2+TC2</x:v>
       </x:c>
       <x:c r="G177" s="63" t="str">
-        <x:v>SUKANTA GHOSH</x:v>
+        <x:v>SHUNMUGA PERUMAL P</x:v>
       </x:c>
     </x:row>
     <x:row r="178" ht="15" hidden="0" customHeight="1">
       <x:c r="A178" s="61" t="str">
-        <x:v>BCSE102P</x:v>
+        <x:v>BITE409L</x:v>
       </x:c>
       <x:c r="B178" s="62" t="str">
-        <x:v>Structured and Object-Oriented Programming Lab</x:v>
+        <x:v>Mobile Application Development</x:v>
       </x:c>
       <x:c r="C178" s="62" t="str">
-        <x:v>LO</x:v>
+        <x:v>TH</x:v>
       </x:c>
       <x:c r="D178" s="107" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E178" s="62" t="str">
-        <x:v>PRP347</x:v>
+        <x:v>SJT824</x:v>
       </x:c>
       <x:c r="F178" s="62" t="str">
-        <x:v>L39+L40+L55+L56</x:v>
+        <x:v>C1+TC1</x:v>
       </x:c>
       <x:c r="G178" s="63" t="str">
-        <x:v>SUKANTA GHOSH</x:v>
+        <x:v>SHUNMUGA PERUMAL P</x:v>
       </x:c>
     </x:row>
     <x:row r="179" ht="15" hidden="0" customHeight="1">
       <x:c r="A179" s="61" t="str">
-        <x:v>BCSE102P</x:v>
+        <x:v>BITE409L</x:v>
       </x:c>
       <x:c r="B179" s="62" t="str">
-        <x:v>Structured and Object-Oriented Programming Lab</x:v>
+        <x:v>Mobile Application Development</x:v>
       </x:c>
       <x:c r="C179" s="62" t="str">
-        <x:v>LO</x:v>
+        <x:v>TH</x:v>
       </x:c>
       <x:c r="D179" s="107" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E179" s="62" t="str">
-        <x:v>PRP138</x:v>
+        <x:v>SJT807</x:v>
       </x:c>
       <x:c r="F179" s="62" t="str">
-        <x:v>L13+L14+L27+L28</x:v>
+        <x:v>C2+TC2</x:v>
       </x:c>
       <x:c r="G179" s="63" t="str">
-        <x:v>SUKANTA GHOSH</x:v>
+        <x:v>JEEVITHA P</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180" ht="15" hidden="0" customHeight="1">
+      <x:c r="A180" s="61" t="str">
+        <x:v>BITE410L</x:v>
+      </x:c>
+      <x:c r="B180" s="62" t="str">
+        <x:v>Machine Learning</x:v>
+      </x:c>
+      <x:c r="C180" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D180" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E180" s="62" t="str">
+        <x:v>SJT103</x:v>
+      </x:c>
+      <x:c r="F180" s="62" t="str">
+        <x:v>E1+TE1</x:v>
+      </x:c>
+      <x:c r="G180" s="63" t="str">
+        <x:v>DHIVYA E</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="15" hidden="0" customHeight="1">
+      <x:c r="A181" s="61" t="str">
+        <x:v>BITE410L</x:v>
+      </x:c>
+      <x:c r="B181" s="62" t="str">
+        <x:v>Machine Learning</x:v>
+      </x:c>
+      <x:c r="C181" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D181" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E181" s="62" t="str">
+        <x:v>SJT109</x:v>
+      </x:c>
+      <x:c r="F181" s="62" t="str">
+        <x:v>E2+TE2</x:v>
+      </x:c>
+      <x:c r="G181" s="63" t="str">
+        <x:v>NIVEDITA S</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" ht="15" hidden="0" customHeight="1">
+      <x:c r="A182" s="61" t="str">
+        <x:v>BITE410L</x:v>
+      </x:c>
+      <x:c r="B182" s="62" t="str">
+        <x:v>Machine Learning</x:v>
+      </x:c>
+      <x:c r="C182" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D182" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E182" s="62" t="str">
+        <x:v>SJT115</x:v>
+      </x:c>
+      <x:c r="F182" s="62" t="str">
+        <x:v>E1+TE1</x:v>
+      </x:c>
+      <x:c r="G182" s="63" t="str">
+        <x:v>KISHORERAJA P C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" ht="15" hidden="0" customHeight="1">
+      <x:c r="A183" s="61" t="str">
+        <x:v>BITE410L</x:v>
+      </x:c>
+      <x:c r="B183" s="62" t="str">
+        <x:v>Machine Learning</x:v>
+      </x:c>
+      <x:c r="C183" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D183" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E183" s="62" t="str">
+        <x:v>SJT125</x:v>
+      </x:c>
+      <x:c r="F183" s="62" t="str">
+        <x:v>E2+TE2</x:v>
+      </x:c>
+      <x:c r="G183" s="63" t="str">
+        <x:v>JAGANNATHAN J</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184" ht="15" hidden="0" customHeight="1">
+      <x:c r="A184" s="61" t="str">
+        <x:v>BITE401L</x:v>
+      </x:c>
+      <x:c r="B184" s="62" t="str">
+        <x:v>Network and Information Security</x:v>
+      </x:c>
+      <x:c r="C184" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D184" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E184" s="62" t="str">
+        <x:v>SJT104</x:v>
+      </x:c>
+      <x:c r="F184" s="62" t="str">
+        <x:v>A1+TA1</x:v>
+      </x:c>
+      <x:c r="G184" s="63" t="str">
+        <x:v>ASIS KUMAR TRIPATHY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" ht="15" hidden="0" customHeight="1">
+      <x:c r="A185" s="61" t="str">
+        <x:v>BITE401L</x:v>
+      </x:c>
+      <x:c r="B185" s="62" t="str">
+        <x:v>Network and Information Security</x:v>
+      </x:c>
+      <x:c r="C185" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D185" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E185" s="62" t="str">
+        <x:v>SJT825</x:v>
+      </x:c>
+      <x:c r="F185" s="62" t="str">
+        <x:v>A2+TA2</x:v>
+      </x:c>
+      <x:c r="G185" s="63" t="str">
+        <x:v>MEENATCHI S</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186" ht="15" hidden="0" customHeight="1">
+      <x:c r="A186" s="61" t="str">
+        <x:v>BITE401L</x:v>
+      </x:c>
+      <x:c r="B186" s="62" t="str">
+        <x:v>Network and Information Security</x:v>
+      </x:c>
+      <x:c r="C186" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D186" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E186" s="62" t="str">
+        <x:v>SJT125</x:v>
+      </x:c>
+      <x:c r="F186" s="62" t="str">
+        <x:v>A1+TA1</x:v>
+      </x:c>
+      <x:c r="G186" s="63" t="str">
+        <x:v>THANGA MARIAPPAN L</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187" ht="15" hidden="0" customHeight="1">
+      <x:c r="A187" s="61" t="str">
+        <x:v>BITE401L</x:v>
+      </x:c>
+      <x:c r="B187" s="62" t="str">
+        <x:v>Network and Information Security</x:v>
+      </x:c>
+      <x:c r="C187" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D187" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E187" s="62" t="str">
+        <x:v>SJTG24</x:v>
+      </x:c>
+      <x:c r="F187" s="62" t="str">
+        <x:v>A2+TA2</x:v>
+      </x:c>
+      <x:c r="G187" s="63" t="str">
+        <x:v>THANGA MARIAPPAN L</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188" ht="15" hidden="0" customHeight="1">
+      <x:c r="A188" s="61" t="str">
+        <x:v>BITE401L</x:v>
+      </x:c>
+      <x:c r="B188" s="62" t="str">
+        <x:v>Network and Information Security</x:v>
+      </x:c>
+      <x:c r="C188" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D188" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E188" s="62" t="str">
+        <x:v>SJT124</x:v>
+      </x:c>
+      <x:c r="F188" s="62" t="str">
+        <x:v>A1+TA1</x:v>
+      </x:c>
+      <x:c r="G188" s="63" t="str">
+        <x:v>MEENATCHI S</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189" ht="15" hidden="0" customHeight="1">
+      <x:c r="A189" s="61" t="str">
+        <x:v>BITE401L</x:v>
+      </x:c>
+      <x:c r="B189" s="62" t="str">
+        <x:v>Network and Information Security</x:v>
+      </x:c>
+      <x:c r="C189" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D189" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E189" s="62" t="str">
+        <x:v>SJT103</x:v>
+      </x:c>
+      <x:c r="F189" s="62" t="str">
+        <x:v>A1+TA1</x:v>
+      </x:c>
+      <x:c r="G189" s="63" t="str">
+        <x:v>SRINIVAS KOPPU</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190" ht="15" hidden="0" customHeight="1">
+      <x:c r="A190" s="61" t="str">
+        <x:v>BITE401L</x:v>
+      </x:c>
+      <x:c r="B190" s="62" t="str">
+        <x:v>Network and Information Security</x:v>
+      </x:c>
+      <x:c r="C190" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D190" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E190" s="62" t="str">
+        <x:v>SJT104</x:v>
+      </x:c>
+      <x:c r="F190" s="62" t="str">
+        <x:v>A2+TA2</x:v>
+      </x:c>
+      <x:c r="G190" s="63" t="str">
+        <x:v>SRINIVAS KOPPU</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" ht="15" hidden="0" customHeight="1">
+      <x:c r="A191" s="61" t="str">
+        <x:v>BITE401L</x:v>
+      </x:c>
+      <x:c r="B191" s="62" t="str">
+        <x:v>Network and Information Security</x:v>
+      </x:c>
+      <x:c r="C191" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D191" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E191" s="62" t="str">
+        <x:v>SJT101</x:v>
+      </x:c>
+      <x:c r="F191" s="62" t="str">
+        <x:v>A2+TA2</x:v>
+      </x:c>
+      <x:c r="G191" s="63" t="str">
+        <x:v>ASIS KUMAR TRIPATHY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192" ht="15" hidden="0" customHeight="1">
+      <x:c r="A192" s="61" t="str">
+        <x:v>BITE402L</x:v>
+      </x:c>
+      <x:c r="B192" s="62" t="str">
+        <x:v>Distributed Computing</x:v>
+      </x:c>
+      <x:c r="C192" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D192" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E192" s="62" t="str">
+        <x:v>SJT709</x:v>
+      </x:c>
+      <x:c r="F192" s="62" t="str">
+        <x:v>B1+TB1</x:v>
+      </x:c>
+      <x:c r="G192" s="63" t="str">
+        <x:v>VANI M P</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193" ht="15" hidden="0" customHeight="1">
+      <x:c r="A193" s="61" t="str">
+        <x:v>BITE402L</x:v>
+      </x:c>
+      <x:c r="B193" s="62" t="str">
+        <x:v>Distributed Computing</x:v>
+      </x:c>
+      <x:c r="C193" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D193" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E193" s="62" t="str">
+        <x:v>SJT707</x:v>
+      </x:c>
+      <x:c r="F193" s="62" t="str">
+        <x:v>B2+TB2</x:v>
+      </x:c>
+      <x:c r="G193" s="63" t="str">
+        <x:v>VANI M P</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194" ht="15" hidden="0" customHeight="1">
+      <x:c r="A194" s="61" t="str">
+        <x:v>BITE402L</x:v>
+      </x:c>
+      <x:c r="B194" s="62" t="str">
+        <x:v>Distributed Computing</x:v>
+      </x:c>
+      <x:c r="C194" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D194" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E194" s="62" t="str">
+        <x:v>SJT807</x:v>
+      </x:c>
+      <x:c r="F194" s="62" t="str">
+        <x:v>B1+TB1</x:v>
+      </x:c>
+      <x:c r="G194" s="63" t="str">
+        <x:v>RATHI R</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195" ht="15" hidden="0" customHeight="1">
+      <x:c r="A195" s="61" t="str">
+        <x:v>BITE402L</x:v>
+      </x:c>
+      <x:c r="B195" s="62" t="str">
+        <x:v>Distributed Computing</x:v>
+      </x:c>
+      <x:c r="C195" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D195" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E195" s="62" t="str">
+        <x:v>SJT802</x:v>
+      </x:c>
+      <x:c r="F195" s="62" t="str">
+        <x:v>B1+TB1</x:v>
+      </x:c>
+      <x:c r="G195" s="63" t="str">
+        <x:v>VENKETESH P</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196" ht="15" hidden="0" customHeight="1">
+      <x:c r="A196" s="61" t="str">
+        <x:v>BITE402L</x:v>
+      </x:c>
+      <x:c r="B196" s="62" t="str">
+        <x:v>Distributed Computing</x:v>
+      </x:c>
+      <x:c r="C196" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D196" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E196" s="62" t="str">
+        <x:v>SJT803</x:v>
+      </x:c>
+      <x:c r="F196" s="62" t="str">
+        <x:v>B2+TB2</x:v>
+      </x:c>
+      <x:c r="G196" s="63" t="str">
+        <x:v>VENKETESH P</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197" ht="15" hidden="0" customHeight="1">
+      <x:c r="A197" s="61" t="str">
+        <x:v>BITE402L</x:v>
+      </x:c>
+      <x:c r="B197" s="62" t="str">
+        <x:v>Distributed Computing</x:v>
+      </x:c>
+      <x:c r="C197" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D197" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E197" s="62" t="str">
+        <x:v>SJT715</x:v>
+      </x:c>
+      <x:c r="F197" s="62" t="str">
+        <x:v>B1+TB1</x:v>
+      </x:c>
+      <x:c r="G197" s="63" t="str">
+        <x:v>SENTHILKUMAR T</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198" ht="15" hidden="0" customHeight="1">
+      <x:c r="A198" s="61" t="str">
+        <x:v>BITE402L</x:v>
+      </x:c>
+      <x:c r="B198" s="62" t="str">
+        <x:v>Distributed Computing</x:v>
+      </x:c>
+      <x:c r="C198" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D198" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E198" s="62" t="str">
+        <x:v>SJT712</x:v>
+      </x:c>
+      <x:c r="F198" s="62" t="str">
+        <x:v>B2+TB2</x:v>
+      </x:c>
+      <x:c r="G198" s="63" t="str">
+        <x:v>MEENATCHI S</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199" ht="15" hidden="0" customHeight="1">
+      <x:c r="A199" s="61" t="str">
+        <x:v>BITE402L</x:v>
+      </x:c>
+      <x:c r="B199" s="62" t="str">
+        <x:v>Distributed Computing</x:v>
+      </x:c>
+      <x:c r="C199" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D199" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E199" s="62" t="str">
+        <x:v>SJT626</x:v>
+      </x:c>
+      <x:c r="F199" s="62" t="str">
+        <x:v>B2+TB2</x:v>
+      </x:c>
+      <x:c r="G199" s="63" t="str">
+        <x:v>BHUVANA S</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200" ht="15" hidden="0" customHeight="1">
+      <x:c r="A200" s="61" t="str">
+        <x:v>BITE411L</x:v>
+      </x:c>
+      <x:c r="B200" s="62" t="str">
+        <x:v>Big Data Analytics</x:v>
+      </x:c>
+      <x:c r="C200" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D200" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E200" s="62" t="str">
+        <x:v>SJTG14</x:v>
+      </x:c>
+      <x:c r="F200" s="62" t="str">
+        <x:v>D1+TD1</x:v>
+      </x:c>
+      <x:c r="G200" s="63" t="str">
+        <x:v>RATHI R</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201" ht="15" hidden="0" customHeight="1">
+      <x:c r="A201" s="61" t="str">
+        <x:v>BITE411L</x:v>
+      </x:c>
+      <x:c r="B201" s="62" t="str">
+        <x:v>Big Data Analytics</x:v>
+      </x:c>
+      <x:c r="C201" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D201" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E201" s="62" t="str">
+        <x:v>SJT824</x:v>
+      </x:c>
+      <x:c r="F201" s="62" t="str">
+        <x:v>D1+TD1</x:v>
+      </x:c>
+      <x:c r="G201" s="63" t="str">
+        <x:v>HARSHITA PATEL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202" ht="15" hidden="0" customHeight="1">
+      <x:c r="A202" s="61" t="str">
+        <x:v>BITE411L</x:v>
+      </x:c>
+      <x:c r="B202" s="62" t="str">
+        <x:v>Big Data Analytics</x:v>
+      </x:c>
+      <x:c r="C202" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D202" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E202" s="62" t="str">
+        <x:v>SJTG16</x:v>
+      </x:c>
+      <x:c r="F202" s="62" t="str">
+        <x:v>D1+TD1</x:v>
+      </x:c>
+      <x:c r="G202" s="63" t="str">
+        <x:v>RAJESH P</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203" ht="15" hidden="0" customHeight="1">
+      <x:c r="A203" s="61" t="str">
+        <x:v>BITE411L</x:v>
+      </x:c>
+      <x:c r="B203" s="62" t="str">
+        <x:v>Big Data Analytics</x:v>
+      </x:c>
+      <x:c r="C203" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D203" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E203" s="62" t="str">
+        <x:v>SJTG24</x:v>
+      </x:c>
+      <x:c r="F203" s="62" t="str">
+        <x:v>D2+TD2</x:v>
+      </x:c>
+      <x:c r="G203" s="63" t="str">
+        <x:v>PRAVEEN KUMAR REDDY M</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" ht="15" hidden="0" customHeight="1">
+      <x:c r="A204" s="61" t="str">
+        <x:v>BITE411L</x:v>
+      </x:c>
+      <x:c r="B204" s="62" t="str">
+        <x:v>Big Data Analytics</x:v>
+      </x:c>
+      <x:c r="C204" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D204" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E204" s="62" t="str">
+        <x:v>SJT825</x:v>
+      </x:c>
+      <x:c r="F204" s="62" t="str">
+        <x:v>D2+TD2</x:v>
+      </x:c>
+      <x:c r="G204" s="63" t="str">
+        <x:v>RATHI R</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205" ht="15" hidden="0" customHeight="1">
+      <x:c r="A205" s="61" t="str">
+        <x:v>BITE411L</x:v>
+      </x:c>
+      <x:c r="B205" s="62" t="str">
+        <x:v>Big Data Analytics</x:v>
+      </x:c>
+      <x:c r="C205" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D205" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E205" s="62" t="str">
+        <x:v>SJT825</x:v>
+      </x:c>
+      <x:c r="F205" s="62" t="str">
+        <x:v>D1+TD1</x:v>
+      </x:c>
+      <x:c r="G205" s="63" t="str">
+        <x:v>CHANDRA MOULISWARAN S</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206" ht="15" hidden="0" customHeight="1">
+      <x:c r="A206" s="61" t="str">
+        <x:v>BITE411L</x:v>
+      </x:c>
+      <x:c r="B206" s="62" t="str">
+        <x:v>Big Data Analytics</x:v>
+      </x:c>
+      <x:c r="C206" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D206" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E206" s="62" t="str">
+        <x:v>SJT824</x:v>
+      </x:c>
+      <x:c r="F206" s="62" t="str">
+        <x:v>D2+TD2</x:v>
+      </x:c>
+      <x:c r="G206" s="63" t="str">
+        <x:v>CHANDRA MOULISWARAN S</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207" ht="15" hidden="0" customHeight="1">
+      <x:c r="A207" s="61" t="str">
+        <x:v>BITE411L</x:v>
+      </x:c>
+      <x:c r="B207" s="62" t="str">
+        <x:v>Big Data Analytics</x:v>
+      </x:c>
+      <x:c r="C207" s="62" t="str">
+        <x:v>TH</x:v>
+      </x:c>
+      <x:c r="D207" s="107" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E207" s="62" t="str">
+        <x:v>SJT823</x:v>
+      </x:c>
+      <x:c r="F207" s="62" t="str">
+        <x:v>D2+TD2</x:v>
+      </x:c>
+      <x:c r="G207" s="63" t="str">
+        <x:v>PADMAKUMARI P</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208" ht="15" hidden="0" customHeight="1">
+      <x:c r="A208" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B208" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C208" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D208" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E208" s="62" t="str">
+        <x:v>SMV218</x:v>
+      </x:c>
+      <x:c r="F208" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G208" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209" ht="15" hidden="0" customHeight="1">
+      <x:c r="A209" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B209" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C209" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D209" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E209" s="62" t="str">
+        <x:v>SMV218</x:v>
+      </x:c>
+      <x:c r="F209" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G209" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210" ht="15" hidden="0" customHeight="1">
+      <x:c r="A210" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B210" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C210" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D210" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E210" s="62" t="str">
+        <x:v>SMV219</x:v>
+      </x:c>
+      <x:c r="F210" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G210" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="211" ht="15" hidden="0" customHeight="1">
+      <x:c r="A211" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B211" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C211" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D211" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E211" s="62" t="str">
+        <x:v>SMV102</x:v>
+      </x:c>
+      <x:c r="F211" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G211" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212" ht="15" hidden="0" customHeight="1">
+      <x:c r="A212" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B212" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C212" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D212" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E212" s="62" t="str">
+        <x:v>CDMM405</x:v>
+      </x:c>
+      <x:c r="F212" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G212" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" ht="15" hidden="0" customHeight="1">
+      <x:c r="A213" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B213" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C213" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D213" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E213" s="62" t="str">
+        <x:v>TT630</x:v>
+      </x:c>
+      <x:c r="F213" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G213" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" ht="15" hidden="0" customHeight="1">
+      <x:c r="A214" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B214" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C214" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D214" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E214" s="62" t="str">
+        <x:v>SJT201</x:v>
+      </x:c>
+      <x:c r="F214" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G214" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215" ht="15" hidden="0" customHeight="1">
+      <x:c r="A215" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B215" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C215" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D215" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E215" s="62" t="str">
+        <x:v>SJT202</x:v>
+      </x:c>
+      <x:c r="F215" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G215" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216" ht="15" hidden="0" customHeight="1">
+      <x:c r="A216" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B216" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C216" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D216" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E216" s="62" t="str">
+        <x:v>SJT204</x:v>
+      </x:c>
+      <x:c r="F216" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G216" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217" ht="15" hidden="0" customHeight="1">
+      <x:c r="A217" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B217" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C217" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D217" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E217" s="62" t="str">
+        <x:v>SJT208</x:v>
+      </x:c>
+      <x:c r="F217" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G217" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218" ht="15" hidden="0" customHeight="1">
+      <x:c r="A218" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B218" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C218" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D218" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E218" s="62" t="str">
+        <x:v>SJT211</x:v>
+      </x:c>
+      <x:c r="F218" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G218" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219" ht="15" hidden="0" customHeight="1">
+      <x:c r="A219" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B219" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C219" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D219" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E219" s="62" t="str">
+        <x:v>SJT211</x:v>
+      </x:c>
+      <x:c r="F219" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G219" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220" ht="15" hidden="0" customHeight="1">
+      <x:c r="A220" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B220" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C220" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D220" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E220" s="62" t="str">
+        <x:v>GDN121</x:v>
+      </x:c>
+      <x:c r="F220" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G220" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221" ht="15" hidden="0" customHeight="1">
+      <x:c r="A221" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B221" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C221" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D221" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E221" s="62" t="str">
+        <x:v>GDN122</x:v>
+      </x:c>
+      <x:c r="F221" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G221" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222" ht="15" hidden="0" customHeight="1">
+      <x:c r="A222" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B222" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C222" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D222" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E222" s="62" t="str">
+        <x:v>GDN107</x:v>
+      </x:c>
+      <x:c r="F222" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G222" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223" ht="15" hidden="0" customHeight="1">
+      <x:c r="A223" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B223" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C223" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D223" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E223" s="62" t="str">
+        <x:v>GDN107</x:v>
+      </x:c>
+      <x:c r="F223" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G223" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224" ht="15" hidden="0" customHeight="1">
+      <x:c r="A224" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B224" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C224" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D224" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E224" s="62" t="str">
+        <x:v>GDN121</x:v>
+      </x:c>
+      <x:c r="F224" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G224" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225" ht="15" hidden="0" customHeight="1">
+      <x:c r="A225" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B225" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C225" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D225" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E225" s="62" t="str">
+        <x:v>SMV219</x:v>
+      </x:c>
+      <x:c r="F225" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G225" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226" ht="15" hidden="0" customHeight="1">
+      <x:c r="A226" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B226" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C226" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D226" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E226" s="62" t="str">
+        <x:v>TT404</x:v>
+      </x:c>
+      <x:c r="F226" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G226" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227" ht="15" hidden="0" customHeight="1">
+      <x:c r="A227" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B227" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C227" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D227" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E227" s="62" t="str">
+        <x:v>SJT204</x:v>
+      </x:c>
+      <x:c r="F227" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G227" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228" ht="15" hidden="0" customHeight="1">
+      <x:c r="A228" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B228" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C228" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D228" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E228" s="62" t="str">
+        <x:v>SJT205</x:v>
+      </x:c>
+      <x:c r="F228" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G228" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229" ht="15" hidden="0" customHeight="1">
+      <x:c r="A229" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B229" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C229" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D229" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E229" s="62" t="str">
+        <x:v>SJT205</x:v>
+      </x:c>
+      <x:c r="F229" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G229" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="230" ht="15" hidden="0" customHeight="1">
+      <x:c r="A230" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B230" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C230" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D230" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E230" s="62" t="str">
+        <x:v>SJT208</x:v>
+      </x:c>
+      <x:c r="F230" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G230" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="231" ht="15" hidden="0" customHeight="1">
+      <x:c r="A231" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B231" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C231" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D231" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E231" s="62" t="str">
+        <x:v>GDN120</x:v>
+      </x:c>
+      <x:c r="F231" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G231" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232" ht="15" hidden="0" customHeight="1">
+      <x:c r="A232" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B232" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C232" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D232" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E232" s="62" t="str">
+        <x:v>GDN122</x:v>
+      </x:c>
+      <x:c r="F232" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G232" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="233" ht="15" hidden="0" customHeight="1">
+      <x:c r="A233" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B233" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C233" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D233" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E233" s="62" t="str">
+        <x:v>SMV102</x:v>
+      </x:c>
+      <x:c r="F233" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G233" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="234" ht="15" hidden="0" customHeight="1">
+      <x:c r="A234" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B234" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C234" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D234" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E234" s="62" t="str">
+        <x:v>TT630</x:v>
+      </x:c>
+      <x:c r="F234" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G234" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="235" ht="15" hidden="0" customHeight="1">
+      <x:c r="A235" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B235" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C235" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D235" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E235" s="62" t="str">
+        <x:v>CDMM405</x:v>
+      </x:c>
+      <x:c r="F235" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G235" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236" ht="15" hidden="0" customHeight="1">
+      <x:c r="A236" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B236" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C236" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D236" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E236" s="62" t="str">
+        <x:v>GDN106</x:v>
+      </x:c>
+      <x:c r="F236" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G236" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="237" ht="15" hidden="0" customHeight="1">
+      <x:c r="A237" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B237" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C237" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D237" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E237" s="62" t="str">
+        <x:v>GDN120</x:v>
+      </x:c>
+      <x:c r="F237" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G237" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238" ht="15" hidden="0" customHeight="1">
+      <x:c r="A238" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B238" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C238" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D238" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E238" s="62" t="str">
+        <x:v>GDN123</x:v>
+      </x:c>
+      <x:c r="F238" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G238" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239" ht="15" hidden="0" customHeight="1">
+      <x:c r="A239" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B239" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C239" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D239" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E239" s="62" t="str">
+        <x:v>TT524</x:v>
+      </x:c>
+      <x:c r="F239" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G239" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240" ht="15" hidden="0" customHeight="1">
+      <x:c r="A240" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B240" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C240" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D240" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E240" s="62" t="str">
+        <x:v>TT531</x:v>
+      </x:c>
+      <x:c r="F240" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G240" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="241" ht="15" hidden="0" customHeight="1">
+      <x:c r="A241" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B241" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C241" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D241" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E241" s="62" t="str">
+        <x:v>TT531</x:v>
+      </x:c>
+      <x:c r="F241" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G241" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242" ht="15" hidden="0" customHeight="1">
+      <x:c r="A242" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B242" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C242" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D242" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E242" s="62" t="str">
+        <x:v>TT404</x:v>
+      </x:c>
+      <x:c r="F242" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G242" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="243" ht="15" hidden="0" customHeight="1">
+      <x:c r="A243" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B243" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C243" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D243" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E243" s="62" t="str">
+        <x:v>SJT201</x:v>
+      </x:c>
+      <x:c r="F243" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G243" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="244" ht="15" hidden="0" customHeight="1">
+      <x:c r="A244" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B244" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C244" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D244" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E244" s="62" t="str">
+        <x:v>SJT202</x:v>
+      </x:c>
+      <x:c r="F244" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G244" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245" ht="15" hidden="0" customHeight="1">
+      <x:c r="A245" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B245" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C245" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D245" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E245" s="62" t="str">
+        <x:v>TT523</x:v>
+      </x:c>
+      <x:c r="F245" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G245" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="246" ht="15" hidden="0" customHeight="1">
+      <x:c r="A246" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B246" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C246" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D246" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E246" s="62" t="str">
+        <x:v>TT523</x:v>
+      </x:c>
+      <x:c r="F246" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G246" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247" ht="15" hidden="0" customHeight="1">
+      <x:c r="A247" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B247" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C247" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D247" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E247" s="62" t="str">
+        <x:v>GDN106</x:v>
+      </x:c>
+      <x:c r="F247" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G247" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248" ht="15" hidden="0" customHeight="1">
+      <x:c r="A248" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B248" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C248" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D248" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E248" s="62" t="str">
+        <x:v>GDN123</x:v>
+      </x:c>
+      <x:c r="F248" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G248" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249" ht="15" hidden="0" customHeight="1">
+      <x:c r="A249" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B249" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C249" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D249" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E249" s="62" t="str">
+        <x:v>TT530</x:v>
+      </x:c>
+      <x:c r="F249" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G249" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250" ht="15" hidden="0" customHeight="1">
+      <x:c r="A250" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B250" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C250" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D250" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E250" s="62" t="str">
+        <x:v>TT530A</x:v>
+      </x:c>
+      <x:c r="F250" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G250" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251" ht="15" hidden="0" customHeight="1">
+      <x:c r="A251" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B251" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C251" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D251" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E251" s="62" t="str">
+        <x:v>TT531A</x:v>
+      </x:c>
+      <x:c r="F251" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G251" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252" ht="15" hidden="0" customHeight="1">
+      <x:c r="A252" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B252" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C252" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D252" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E252" s="62" t="str">
+        <x:v>TT531A</x:v>
+      </x:c>
+      <x:c r="F252" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G252" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="253" ht="15" hidden="0" customHeight="1">
+      <x:c r="A253" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B253" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C253" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D253" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E253" s="62" t="str">
+        <x:v>TT504</x:v>
+      </x:c>
+      <x:c r="F253" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G253" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="254" ht="15" hidden="0" customHeight="1">
+      <x:c r="A254" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B254" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C254" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D254" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E254" s="62" t="str">
+        <x:v>TT504</x:v>
+      </x:c>
+      <x:c r="F254" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G254" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="255" ht="15" hidden="0" customHeight="1">
+      <x:c r="A255" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B255" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C255" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D255" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E255" s="62" t="str">
+        <x:v>TT524</x:v>
+      </x:c>
+      <x:c r="F255" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G255" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="256" ht="15" hidden="0" customHeight="1">
+      <x:c r="A256" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B256" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C256" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D256" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E256" s="62" t="str">
+        <x:v>TT530A</x:v>
+      </x:c>
+      <x:c r="F256" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G256" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="257" ht="15" hidden="0" customHeight="1">
+      <x:c r="A257" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B257" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C257" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D257" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E257" s="62" t="str">
+        <x:v>TT434</x:v>
+      </x:c>
+      <x:c r="F257" s="62" t="str">
+        <x:v>F1+TF1</x:v>
+      </x:c>
+      <x:c r="G257" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="258" ht="15" hidden="0" customHeight="1">
+      <x:c r="A258" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B258" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C258" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D258" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E258" s="62" t="str">
+        <x:v>TT530</x:v>
+      </x:c>
+      <x:c r="F258" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G258" s="63" t="str">
+        <x:v>ETHNUS (APT)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="259" ht="15" hidden="0" customHeight="1">
+      <x:c r="A259" s="61" t="str">
+        <x:v>BSTS302P</x:v>
+      </x:c>
+      <x:c r="B259" s="62" t="str">
+        <x:v>Advanced Competitive Coding - II</x:v>
+      </x:c>
+      <x:c r="C259" s="62" t="str">
+        <x:v>SS</x:v>
+      </x:c>
+      <x:c r="D259" s="107" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E259" s="62" t="str">
+        <x:v>TT434</x:v>
+      </x:c>
+      <x:c r="F259" s="62" t="str">
+        <x:v>F2+TF2</x:v>
+      </x:c>
+      <x:c r="G259" s="63" t="str">
+        <x:v>FACE (APT)</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9479282cab684baf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0c54b304b574bec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>